<commit_message>
Update package dependencies, enhance evaluation results, and refine model outputs
</commit_message>
<xml_diff>
--- a/outputs/employee_data_pivot.xlsx
+++ b/outputs/employee_data_pivot.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pivot" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -471,7 +471,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Years</t>
+          <t>YearsWithCompany</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update models.json to switch to GitHub Copilot's Claude Sonnet 4.6, enhance contract document with detailed executive summary, and normalize invoice CSV format. Additionally, several binary files were updated, and multiple image files were deleted.
</commit_message>
<xml_diff>
--- a/outputs/employee_data_pivot.xlsx
+++ b/outputs/employee_data_pivot.xlsx
@@ -2,12 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pivot" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -17,11 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,14 +27,42 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+        <bgColor rgb="00BDD7EE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -50,24 +74,40 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -430,48 +470,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>EmployeeID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Salary</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>PerformanceScore</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>IsRemote</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>YearsWithCompany</t>
         </is>
       </c>
     </row>
@@ -494,17 +529,18 @@
       <c r="D2" t="n">
         <v>133810</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>43677</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2019-07-31</t>
+        </is>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>6.620123203285421</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -526,17 +562,18 @@
       <c r="D3" t="n">
         <v>82098</v>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>43448</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2018-12-14</t>
+        </is>
       </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>7.247091033538672</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -558,17 +595,18 @@
       <c r="D4" t="n">
         <v>138696</v>
       </c>
-      <c r="E4" s="2" t="n">
-        <v>42789</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2017-02-23</t>
+        </is>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>9.051334702258726</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -590,17 +628,18 @@
       <c r="D5" t="n">
         <v>54165</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>43844</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2020-01-14</t>
+        </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>6.16290212183436</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -622,17 +661,18 @@
       <c r="D6" t="n">
         <v>80495</v>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>42871</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2017-05-16</t>
+        </is>
       </c>
       <c r="F6" t="n">
         <v>5</v>
       </c>
-      <c r="G6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>8.826830937713895</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -654,17 +694,18 @@
       <c r="D7" t="n">
         <v>123563</v>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>43498</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2019-02-02</t>
+        </is>
       </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
-      <c r="G7" t="b">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>7.110198494182067</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -686,17 +727,18 @@
       <c r="D8" t="n">
         <v>78893</v>
       </c>
-      <c r="E8" s="2" t="n">
-        <v>42986</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2017-09-08</t>
+        </is>
       </c>
       <c r="F8" t="n">
         <v>5</v>
       </c>
-      <c r="G8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>8.511978097193703</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -718,17 +760,18 @@
       <c r="D9" t="n">
         <v>50851</v>
       </c>
-      <c r="E9" s="2" t="n">
-        <v>43579</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2019-04-24</t>
+        </is>
       </c>
       <c r="F9" t="n">
         <v>4</v>
       </c>
-      <c r="G9" t="b">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>6.888432580424367</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -750,17 +793,18 @@
       <c r="D10" t="n">
         <v>86421</v>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>43587</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2019-05-02</t>
+        </is>
       </c>
       <c r="F10" t="n">
         <v>2</v>
       </c>
-      <c r="G10" t="b">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>6.86652977412731</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -782,17 +826,18 @@
       <c r="D11" t="n">
         <v>63396</v>
       </c>
-      <c r="E11" s="2" t="n">
-        <v>43716</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2019-09-08</t>
+        </is>
       </c>
       <c r="F11" t="n">
         <v>4</v>
       </c>
-      <c r="G11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>6.513347022587269</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -814,17 +859,18 @@
       <c r="D12" t="n">
         <v>97052</v>
       </c>
-      <c r="E12" s="2" t="n">
-        <v>45361</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2024-03-10</t>
+        </is>
       </c>
       <c r="F12" t="n">
         <v>5</v>
       </c>
-      <c r="G12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2.009582477754962</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -846,17 +892,18 @@
       <c r="D13" t="n">
         <v>55695</v>
       </c>
-      <c r="E13" s="2" t="n">
-        <v>45125</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2023-07-18</t>
+        </is>
       </c>
       <c r="F13" t="n">
         <v>5</v>
       </c>
-      <c r="G13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" t="n">
-        <v>2.655715263518138</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -878,17 +925,18 @@
       <c r="D14" t="n">
         <v>99615</v>
       </c>
-      <c r="E14" s="2" t="n">
-        <v>45904</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
       </c>
       <c r="F14" t="n">
         <v>5</v>
       </c>
-      <c r="G14" t="b">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.5229295003422314</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -910,17 +958,18 @@
       <c r="D15" t="n">
         <v>132397</v>
       </c>
-      <c r="E15" s="2" t="n">
-        <v>44799</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2022-08-26</t>
+        </is>
       </c>
       <c r="F15" t="n">
         <v>3</v>
       </c>
-      <c r="G15" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" t="n">
-        <v>3.548254620123203</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -942,17 +991,18 @@
       <c r="D16" t="n">
         <v>142349</v>
       </c>
-      <c r="E16" s="2" t="n">
-        <v>45923</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-09-23</t>
+        </is>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="G16" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.4709103353867214</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -974,17 +1024,18 @@
       <c r="D17" t="n">
         <v>87930</v>
       </c>
-      <c r="E17" s="2" t="n">
-        <v>45902</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
       </c>
       <c r="F17" t="n">
         <v>2</v>
       </c>
-      <c r="G17" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.5284052019164955</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1006,17 +1057,18 @@
       <c r="D18" t="n">
         <v>99823</v>
       </c>
-      <c r="E18" s="2" t="n">
-        <v>45496</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2024-07-23</t>
+        </is>
       </c>
       <c r="F18" t="n">
         <v>4</v>
       </c>
-      <c r="G18" t="b">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>1.639972621492129</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1038,17 +1090,18 @@
       <c r="D19" t="n">
         <v>71319</v>
       </c>
-      <c r="E19" s="2" t="n">
-        <v>45307</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2024-01-16</t>
+        </is>
       </c>
       <c r="F19" t="n">
         <v>3</v>
       </c>
-      <c r="G19" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" t="n">
-        <v>2.157426420260096</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1070,17 +1123,18 @@
       <c r="D20" t="n">
         <v>137841</v>
       </c>
-      <c r="E20" s="2" t="n">
-        <v>45519</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2024-08-15</t>
+        </is>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
-      <c r="G20" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1.57700205338809</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1102,17 +1156,18 @@
       <c r="D21" t="n">
         <v>120010</v>
       </c>
-      <c r="E21" s="2" t="n">
-        <v>45564</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2024-09-29</t>
+        </is>
       </c>
       <c r="F21" t="n">
         <v>2</v>
       </c>
-      <c r="G21" t="b">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1.453798767967146</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1134,17 +1189,18 @@
       <c r="D22" t="n">
         <v>99735</v>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>45513</v>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2024-08-09</t>
+        </is>
       </c>
       <c r="F22" t="n">
         <v>5</v>
       </c>
-      <c r="G22" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" t="n">
-        <v>1.593429158110883</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1166,17 +1222,18 @@
       <c r="D23" t="n">
         <v>139733</v>
       </c>
-      <c r="E23" s="2" t="n">
-        <v>45401</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2024-04-19</t>
+        </is>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
-      <c r="G23" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" t="n">
-        <v>1.900068446269678</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1198,17 +1255,18 @@
       <c r="D24" t="n">
         <v>54207</v>
       </c>
-      <c r="E24" s="2" t="n">
-        <v>45419</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2024-05-07</t>
+        </is>
       </c>
       <c r="F24" t="n">
         <v>4</v>
       </c>
-      <c r="G24" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>1.850787132101301</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1230,17 +1288,18 @@
       <c r="D25" t="n">
         <v>58675</v>
       </c>
-      <c r="E25" s="2" t="n">
-        <v>45633</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2024-12-07</t>
+        </is>
       </c>
       <c r="F25" t="n">
         <v>5</v>
       </c>
-      <c r="G25" t="b">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>1.264887063655031</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1262,21 +1321,22 @@
       <c r="D26" t="n">
         <v>77869</v>
       </c>
-      <c r="E26" s="2" t="n">
-        <v>44723</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2022-06-11</t>
+        </is>
       </c>
       <c r="F26" t="n">
         <v>4</v>
       </c>
-      <c r="G26" t="b">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>3.756331279945243</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1286,8 +1346,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1295,76 +1361,116 @@
           <t>Department</t>
         </is>
       </c>
-      <c r="B1" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="b">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>IsRemote: TRUE</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>IsRemote: FALSE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+      <c r="C4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D5" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2</v>
+      <c r="D6" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>